<commit_message>
update plots and include no CO2
</commit_message>
<xml_diff>
--- a/Plotting/production_shares_ammonia.xlsx
+++ b/Plotting/production_shares_ammonia.xlsx
@@ -504,21 +504,21 @@
       <c r="G2" s="1" t="n"/>
       <c r="H2" s="1" t="inlineStr">
         <is>
-          <t>MPWemission</t>
+          <t>noCO2electrolysis</t>
         </is>
       </c>
       <c r="I2" s="1" t="n"/>
       <c r="J2" s="1" t="n"/>
       <c r="K2" s="1" t="inlineStr">
         <is>
-          <t>OptBIO</t>
+          <t>MPWemission</t>
         </is>
       </c>
       <c r="L2" s="1" t="n"/>
       <c r="M2" s="1" t="n"/>
       <c r="N2" s="1" t="inlineStr">
         <is>
-          <t>noCO2electrolysis</t>
+          <t>OptBIO</t>
         </is>
       </c>
       <c r="O2" s="1" t="n"/>
@@ -735,31 +735,31 @@
         <v>1209392.130763266</v>
       </c>
       <c r="H7" t="n">
+        <v>990560.1484299452</v>
+      </c>
+      <c r="I7" t="n">
+        <v>432361.1672976832</v>
+      </c>
+      <c r="J7" t="n">
+        <v>8900.097826784262</v>
+      </c>
+      <c r="K7" t="n">
         <v>1003302.28224</v>
       </c>
-      <c r="I7" t="n">
+      <c r="L7" t="n">
         <v>999880.50282332</v>
       </c>
-      <c r="J7" t="n">
+      <c r="M7" t="n">
         <v>1010914.192579916</v>
       </c>
-      <c r="K7" t="n">
+      <c r="N7" t="n">
         <v>1003302.282239998</v>
       </c>
-      <c r="L7" t="n">
+      <c r="O7" t="n">
         <v>991969.1294183502</v>
       </c>
-      <c r="M7" t="n">
+      <c r="P7" t="n">
         <v>997933.3467806721</v>
-      </c>
-      <c r="N7" t="n">
-        <v>990560.1484299452</v>
-      </c>
-      <c r="O7" t="n">
-        <v>432361.1672976832</v>
-      </c>
-      <c r="P7" t="n">
-        <v>8900.097826784262</v>
       </c>
     </row>
     <row r="8">
@@ -787,31 +787,31 @@
         <v>605757.6457301588</v>
       </c>
       <c r="H8" t="n">
-        <v>0</v>
+        <v>118878.6504658565</v>
       </c>
       <c r="I8" t="n">
-        <v>0</v>
+        <v>677077.6315981238</v>
       </c>
       <c r="J8" t="n">
+        <v>1120446.693460911</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" t="n">
         <v>4109.032718056557</v>
       </c>
-      <c r="K8" t="n">
-        <v>0</v>
-      </c>
-      <c r="L8" t="n">
+      <c r="N8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" t="n">
         <v>17960.49100618666</v>
       </c>
-      <c r="M8" t="n">
+      <c r="P8" t="n">
         <v>1507.357148631683</v>
-      </c>
-      <c r="N8" t="n">
-        <v>118878.6504658565</v>
-      </c>
-      <c r="O8" t="n">
-        <v>677077.6315981238</v>
-      </c>
-      <c r="P8" t="n">
-        <v>1120446.693460911</v>
       </c>
     </row>
     <row r="9">

</xml_diff>